<commit_message>
Primera atestación real Human Approval (AMS); RE-043.2: Cajas/Proyecciones ya no se leen como patrimonios. CONSTITUTION v1.8, governance v1.91
</commit_message>
<xml_diff>
--- a/data/raw/human_approval_attestations.xlsx
+++ b/data/raw/human_approval_attestations.xlsx
@@ -18,8 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="7">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -63,6 +66,11 @@
       <color rgb="FF0000FF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -103,7 +111,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -174,6 +182,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -605,10 +620,29 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="23" t="n"/>
-      <c r="C5" s="23" t="n"/>
-      <c r="D5" s="23" t="n"/>
+      <c r="A5" s="24" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>Deploy Aggressively</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>Primera atestación registrada.</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
       <c r="A6" s="23" t="n"/>

</xml_diff>

<commit_message>
Primera atestación real Human Approval en AML (Conserve, vigente de inmediato). CONSTITUTION v1.9, governance v1.92
</commit_message>
<xml_diff>
--- a/data/raw/human_approval_attestations.xlsx
+++ b/data/raw/human_approval_attestations.xlsx
@@ -19,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -111,7 +111,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -182,13 +182,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -620,7 +623,7 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
-      <c r="A5" s="24" t="n">
+      <c r="A5" s="27" t="n">
         <v>46247</v>
       </c>
       <c r="B5" s="25" t="inlineStr">
@@ -809,10 +812,29 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="12">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="23" t="n"/>
-      <c r="C5" s="23" t="n"/>
-      <c r="D5" s="23" t="n"/>
+      <c r="A5" s="27" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>Conserve</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>Primera atestación registrada.</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
       <c r="A6" s="23" t="n"/>

</xml_diff>